<commit_message>
feat: added Combined Method Code
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!!Self\Pt1\domain-adapation-main\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3789DAE3-44C8-48FD-9832-0194BBD273E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A07243B-E9BF-4316-9967-7E4A8CCDA241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
   <si>
     <t>SOURCE</t>
   </si>
@@ -79,6 +79,12 @@
   </si>
   <si>
     <t>0.8292</t>
+  </si>
+  <si>
+    <t>DANN +  Adapter</t>
+  </si>
+  <si>
+    <t>DANN + Adapter + Pretraining(Target)</t>
   </si>
 </sst>
 </file>
@@ -302,13 +308,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>189707</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>65322</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -346,13 +352,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>612913</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>565192</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>49696</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -652,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K15"/>
+  <dimension ref="B2:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.42578125" customWidth="1"/>
@@ -773,52 +779,122 @@
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="C6" s="4">
+        <v>0.91620000000000001</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0.91169999999999995</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0.91620000000000001</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.91320000000000001</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0.81869999999999998</v>
+      </c>
+      <c r="H6" s="8">
+        <v>0.84930000000000005</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0.81869999999999998</v>
+      </c>
+      <c r="J6" s="8">
+        <v>0.81469999999999998</v>
+      </c>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0.91649999999999998</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0.91279999999999994</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.91649999999999998</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.91420000000000001</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0.83389999999999997</v>
+      </c>
+      <c r="H7" s="8">
+        <v>0.86009999999999998</v>
+      </c>
+      <c r="I7" s="8">
+        <v>0.83389999999999997</v>
+      </c>
+      <c r="J7" s="8">
+        <v>0.83079999999999998</v>
+      </c>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0.90039999999999998</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0.90069999999999995</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.90039999999999998</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0.90039999999999998</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0.86660000000000004</v>
+      </c>
+      <c r="H8" s="8">
+        <v>0.86670000000000003</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0.86660000000000004</v>
+      </c>
+      <c r="J8" s="8">
+        <v>0.86660000000000004</v>
+      </c>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="K9" s="2"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="3"/>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" t="s">
-        <v>8</v>
-      </c>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -826,6 +902,12 @@
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17" spans="11:11" x14ac:dyDescent="0.25">
+      <c r="K17" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Feat: Updated adapter, matching config and datasets as others
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -5,27 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\nlp-unsupervised-domain-adaptation\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01 Projects\Uni\Pre Thesis\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD58278-44E3-4909-AE65-CB94B2515618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099E481F-CB06-4FEF-95BF-2DBDA113C101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>SOURCE</t>
   </si>
@@ -60,12 +71,6 @@
     <t>NOTES</t>
   </si>
   <si>
-    <t>- Target accuracy lebih tinggi dari source (90.04% vs 88.76%), pola konsisten dengan Pretraining. Namun class negative di target domain sangat lemah (F1: 0.66) vs positive (F1: 0.94)
--&gt; kemungkinan karena imbalance di target test set (6637 pos vs 1032 neg).
-- MMD loss stabil di 0.382–0.385, domain adapter konvergen tapi gap source-target masih ada.
-Overall sedikit di bawah Pretraining, tapi hanya melatih ~1.83% parameter.</t>
-  </si>
-  <si>
     <t>0.8613</t>
   </si>
   <si>
@@ -85,6 +90,13 @@
   </si>
   <si>
     <t>Updated CoastSent + Lazada</t>
+  </si>
+  <si>
+    <t>Adapter V2</t>
+  </si>
+  <si>
+    <t>Updated CoastSent + Lazada
+Low F1 (0.6881)-&gt; due to a large domain gap between coastal tourism reviews and e-commerce product reviews, compounded by label noise in Lazada where rating 3 is ambiguously labeled negative, and limited MMD adaptation capacity to bridge such a significant domain shift.</t>
   </si>
 </sst>
 </file>
@@ -230,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -252,9 +264,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -348,16 +357,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>612913</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2000</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>565192</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>49696</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>88387</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>59121</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -380,8 +389,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4265543" y="2476500"/>
-          <a:ext cx="4242671" cy="5193196"/>
+          <a:off x="4265259" y="2286000"/>
+          <a:ext cx="2530042" cy="3107121"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>124240</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>124568</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8F13B95-3F00-3903-2FE9-582E4F087DC6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4265544" y="5715000"/>
+          <a:ext cx="3801718" cy="3363068"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -656,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K16"/>
+  <dimension ref="B2:K30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.42578125" customWidth="1"/>
@@ -664,27 +717,27 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="14" t="s">
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="17" t="s">
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="16" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="10"/>
+      <c r="B3" s="9"/>
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
@@ -709,68 +762,68 @@
       <c r="J3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="17"/>
+      <c r="K3" s="16"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="H4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>15</v>
-      </c>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="2:11" ht="165" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" ht="120" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="4">
-        <v>0.88759999999999994</v>
+        <v>0.87450000000000006</v>
       </c>
       <c r="D5" s="4">
-        <v>0.89290000000000003</v>
+        <v>0.87690000000000001</v>
       </c>
       <c r="E5" s="4">
-        <v>0.88759999999999994</v>
+        <v>0.87450000000000006</v>
       </c>
       <c r="F5" s="4">
-        <v>0.88800000000000001</v>
+        <v>0.87439999999999996</v>
       </c>
       <c r="G5" s="7">
-        <v>0.90039999999999998</v>
+        <v>0.6986</v>
       </c>
       <c r="H5" s="7">
-        <v>0.90900000000000003</v>
+        <v>0.72929999999999995</v>
       </c>
       <c r="I5" s="7">
-        <v>0.90039999999999998</v>
+        <v>0.6986</v>
       </c>
       <c r="J5" s="7">
-        <v>0.90390000000000004</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>11</v>
+        <v>0.68810000000000004</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
@@ -802,12 +855,12 @@
         <v>0.81789999999999996</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="4">
         <v>0.97089999999999999</v>
@@ -834,12 +887,12 @@
         <v>0.82599999999999996</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="4">
         <v>0.98129999999999995</v>
@@ -866,7 +919,7 @@
         <v>0.85240000000000005</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
@@ -898,6 +951,11 @@
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K16" s="2"/>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
feat: added DAPT+ADAPTER code
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01 Projects\Uni\Pre Thesis\nlp-unsupervised-domain-adaptation\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{099E481F-CB06-4FEF-95BF-2DBDA113C101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9939065-901D-45AB-8289-EA2B427D3F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>SOURCE</t>
   </si>
@@ -97,6 +95,15 @@
   <si>
     <t>Updated CoastSent + Lazada
 Low F1 (0.6881)-&gt; due to a large domain gap between coastal tourism reviews and e-commerce product reviews, compounded by label noise in Lazada where rating 3 is ambiguously labeled negative, and limited MMD adaptation capacity to bridge such a significant domain shift.</t>
+  </si>
+  <si>
+    <t>DAPT + Adapter</t>
+  </si>
+  <si>
+    <t>CoastSent + Lazada</t>
+  </si>
+  <si>
+    <t>Fine Tune IndoBERT (ID-CoastSent)</t>
   </si>
 </sst>
 </file>
@@ -242,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -265,32 +272,38 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -315,13 +328,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>189707</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>65322</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -359,13 +372,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>2000</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>88387</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>59121</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -403,13 +416,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>1</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>124240</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>49</xdr:row>
       <xdr:rowOff>124568</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -709,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K30"/>
+  <dimension ref="B2:K32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.42578125" customWidth="1"/>
@@ -717,27 +730,27 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="13" t="s">
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="16" t="s">
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="17" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="9"/>
+      <c r="B3" s="10"/>
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
@@ -762,129 +775,127 @@
       <c r="J3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="16"/>
+      <c r="K3" s="17"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0.90969999999999995</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.91059999999999997</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.90969999999999995</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.90969999999999995</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0.72940000000000005</v>
+      </c>
+      <c r="H4" s="7">
+        <v>0.76829999999999998</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0.72940000000000005</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0.71909999999999996</v>
+      </c>
+      <c r="K4" s="8"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="2:11" ht="120" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="2:11" ht="120" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C6" s="4">
         <v>0.87450000000000006</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D6" s="4">
         <v>0.87690000000000001</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E6" s="4">
         <v>0.87450000000000006</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F6" s="4">
         <v>0.87439999999999996</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G6" s="7">
         <v>0.6986</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H6" s="7">
         <v>0.72929999999999995</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I6" s="7">
         <v>0.6986</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J6" s="7">
         <v>0.68810000000000004</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.97519999999999996</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0.97519999999999996</v>
-      </c>
-      <c r="E6" s="4">
-        <v>0.97519999999999996</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0.97519999999999996</v>
-      </c>
-      <c r="G6" s="7">
-        <v>0.81830000000000003</v>
-      </c>
-      <c r="H6" s="7">
-        <v>0.82069999999999999</v>
-      </c>
-      <c r="I6" s="7">
-        <v>0.81830000000000003</v>
-      </c>
-      <c r="J6" s="7">
-        <v>0.81789999999999996</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4">
-        <v>0.97089999999999999</v>
+        <v>0.97519999999999996</v>
       </c>
       <c r="D7" s="4">
-        <v>0.97089999999999999</v>
+        <v>0.97519999999999996</v>
       </c>
       <c r="E7" s="4">
-        <v>0.97089999999999999</v>
+        <v>0.97519999999999996</v>
       </c>
       <c r="F7" s="4">
-        <v>0.97089999999999999</v>
+        <v>0.97519999999999996</v>
       </c>
       <c r="G7" s="7">
-        <v>0.82609999999999995</v>
+        <v>0.81830000000000003</v>
       </c>
       <c r="H7" s="7">
-        <v>0.8266</v>
+        <v>0.82069999999999999</v>
       </c>
       <c r="I7" s="7">
-        <v>0.82609999999999995</v>
+        <v>0.81830000000000003</v>
       </c>
       <c r="J7" s="7">
-        <v>0.82599999999999996</v>
+        <v>0.81789999999999996</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>17</v>
@@ -892,58 +903,116 @@
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0.86950000000000005</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0.86960000000000004</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.86950000000000005</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0.86950000000000005</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0.82120000000000004</v>
+      </c>
+      <c r="H8" s="7">
+        <v>0.82140000000000002</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0.82120000000000004</v>
+      </c>
+      <c r="J8" s="7">
+        <v>0.82120000000000004</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0.97089999999999999</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0.97089999999999999</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0.97089999999999999</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0.97089999999999999</v>
+      </c>
+      <c r="G9" s="7">
+        <v>0.82609999999999995</v>
+      </c>
+      <c r="H9" s="7">
+        <v>0.8266</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0.82609999999999995</v>
+      </c>
+      <c r="J9" s="7">
+        <v>0.82599999999999996</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C10" s="4">
         <v>0.98129999999999995</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D10" s="4">
         <v>0.98129999999999995</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E10" s="4">
         <v>0.98129999999999995</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F10" s="4">
         <v>0.98129999999999995</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G10" s="7">
         <v>0.85240000000000005</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H10" s="7">
         <v>0.85250000000000004</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I10" s="7">
         <v>0.85240000000000005</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J10" s="7">
         <v>0.85240000000000005</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="K10" s="2"/>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" t="s">
-        <v>8</v>
-      </c>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
@@ -952,8 +1021,14 @@
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="K16" s="2"/>
     </row>
-    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E30" t="s">
+    <row r="17" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="K18" s="2"/>
+    </row>
+    <row r="32" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Updated Adapter Notes
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\nlp-unsupervised-domain-adaptation\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01 Projects\Uni\Pre Thesis\nlp-unsupervised-domain-adaptation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9939065-901D-45AB-8289-EA2B427D3F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B62195-7B26-48D8-B29D-2174AB6F0DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -93,17 +93,17 @@
     <t>Adapter V2</t>
   </si>
   <si>
+    <t>DAPT + Adapter</t>
+  </si>
+  <si>
+    <t>CoastSent + Lazada</t>
+  </si>
+  <si>
+    <t>Fine Tune IndoBERT (ID-CoastSent)</t>
+  </si>
+  <si>
     <t>Updated CoastSent + Lazada
-Low F1 (0.6881)-&gt; due to a large domain gap between coastal tourism reviews and e-commerce product reviews, compounded by label noise in Lazada where rating 3 is ambiguously labeled negative, and limited MMD adaptation capacity to bridge such a significant domain shift.</t>
-  </si>
-  <si>
-    <t>DAPT + Adapter</t>
-  </si>
-  <si>
-    <t>CoastSent + Lazada</t>
-  </si>
-  <si>
-    <t>Fine Tune IndoBERT (ID-CoastSent)</t>
+Uses only MMD for domain alignment, which minimizes feature distribution distances without adversarial training, making it insufficient to bridge the large domain gap between tourism and e-commerce reviews</t>
   </si>
 </sst>
 </file>
@@ -275,6 +275,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -301,9 +304,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -723,34 +723,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:K32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
-    <col min="11" max="11" width="47.28515625" customWidth="1"/>
+    <col min="2" max="2" width="36.44140625" customWidth="1"/>
+    <col min="11" max="11" width="47.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="9" t="s">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="14" t="s">
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="17" t="s">
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="10"/>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B3" s="11"/>
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
@@ -775,11 +775,11 @@
       <c r="J3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="17"/>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="18" t="s">
-        <v>22</v>
+      <c r="K3" s="18"/>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B4" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C4" s="4">
         <v>0.90969999999999995</v>
@@ -807,7 +807,7 @@
       </c>
       <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
@@ -837,7 +837,7 @@
       </c>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="2:11" ht="120" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
@@ -866,10 +866,10 @@
         <v>0.68810000000000004</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -901,9 +901,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="4">
         <v>0.86950000000000005</v>
@@ -930,10 +930,10 @@
         <v>0.82120000000000004</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>15</v>
       </c>
@@ -965,7 +965,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
@@ -997,16 +997,16 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>7</v>
       </c>
@@ -1015,19 +1015,19 @@
       </c>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:11" x14ac:dyDescent="0.3">
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:11" x14ac:dyDescent="0.3">
       <c r="K18" s="2"/>
     </row>
-    <row r="32" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="5:11" x14ac:dyDescent="0.3">
       <c r="E32" t="s">
         <v>18</v>
       </c>

</xml_diff>

<commit_message>
feat: updated pretraining result
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\!!Self\Pt1\domain-adapation-main\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E317C76-7210-45F6-955E-158B8F562DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE0FEF19-BCB3-4737-B929-82B14063D178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
   <si>
     <t>SOURCE</t>
   </si>
@@ -94,19 +94,16 @@
 Uses only MMD for domain alignment, which minimizes feature distribution distances without adversarial training, making it insufficient to bridge the large domain gap between tourism and e-commerce reviews</t>
   </si>
   <si>
-    <t>0.9147</t>
-  </si>
-  <si>
-    <t>0.9149</t>
-  </si>
-  <si>
     <t>0.8479</t>
   </si>
   <si>
-    <t>0.8471</t>
-  </si>
-  <si>
-    <t>0.8470</t>
+    <t>0.9715</t>
+  </si>
+  <si>
+    <t>0.9175</t>
+  </si>
+  <si>
+    <t>0.8477</t>
   </si>
 </sst>
 </file>
@@ -329,50 +326,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>189707</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>65322</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BD061C5-5F61-46BA-BE72-3A17AC0D13C4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="654844" y="2524125"/>
-          <a:ext cx="3178176" cy="5161197"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>2000</xdr:colOff>
       <xdr:row>14</xdr:row>
@@ -398,7 +351,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -442,7 +395,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -451,6 +404,50 @@
         <a:xfrm>
           <a:off x="4265544" y="5715000"/>
           <a:ext cx="3801718" cy="3363068"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>28341</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>21981</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{41C3969E-A55E-1DFE-05EF-405C9F8DABB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="608135" y="3810000"/>
+          <a:ext cx="3069014" cy="1355481"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -815,28 +812,28 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>22</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>22</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>13</v>

</xml_diff>